<commit_message>
Referencias: motivo de cierre tras carga y ajustes de UI
- Referencias: resuelve la descripcion del motivo de cierre desde el
  catalogo tras procesar el archivo (columna Motivo de cierre visible).
- Informe Referencia: reacomoda filtros (switch "Solo con saldo" y boton
  a segunda fila).
- Actualiza plantilla Formato_Cancelaciones.xlsx.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Formato_Cancelaciones.xlsx
+++ b/public/Formato_Cancelaciones.xlsx
@@ -1,31 +1,43 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ekrontech\portal-govi\public\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C039721-0C55-48AA-A23F-E73A2D94B8D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F8356781-6220-4F11-9D9A-9076419060FE}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
-</workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Hojas de cálculo</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>Hoja1</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
+</file>
+
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Local Admin</dc:creator>
+  <cp:lastModifiedBy>Local Admin</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-19T23:11:16Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-20T15:33:58Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>referencia</t>
   </si>
@@ -38,10 +50,13 @@
   <si>
     <t>aduana</t>
   </si>
+  <si>
+    <t>Motivo de cierre</t>
+  </si>
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -91,20 +106,21 @@
 </styleSheet>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E690729-9814-4DA5-A3F7-256649D7CA3E}" name="Tabla1" displayName="Tabla1" ref="A1:D500" totalsRowShown="0">
-  <autoFilter ref="A1:D500" xr:uid="{2E690729-9814-4DA5-A3F7-256649D7CA3E}"/>
-  <tableColumns count="4">
+<file path=xl\tables\table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E690729-9814-4DA5-A3F7-256649D7CA3E}" name="Tabla1" displayName="Tabla1" ref="A1:E500" totalsRowShown="0">
+  <autoFilter ref="A1:E500" xr:uid="{2E690729-9814-4DA5-A3F7-256649D7CA3E}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{E6557AB6-CF94-4642-B33B-19BF0F289DFD}" name="referencia"/>
     <tableColumn id="2" xr3:uid="{C75042B8-0B46-4A1F-806E-B31C8FE9CA20}" name="estatus"/>
     <tableColumn id="3" xr3:uid="{47690881-797B-4BC5-8CD1-DED9D907931C}" name="pedimento"/>
     <tableColumn id="4" xr3:uid="{9864D4D0-E4CF-44BD-91B9-35FFB32D7E5E}" name="aduana"/>
+    <tableColumn id="5" name="Motivo de cierre"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -399,9 +415,34 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ekrontech\portal-govi\public\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C039721-0C55-48AA-A23F-E73A2D94B8D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F8356781-6220-4F11-9D9A-9076419060FE}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89048D51-76BE-4CD4-9188-9F493A0228F8}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E500"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -421,8 +462,16 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E500">
+      <formula1>"Complementaria incobrable,Diferenciación de impuestos,Multas,Tipo de cambio,Error en registro de IVA,Saldo menor de 300,Gasto no cobrado (Facturación),Facturado Correctamente"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>